<commit_message>
Enable auto-wrapping and dynamic row height for descriptions, make stamps transparent in PO and MR templates
</commit_message>
<xml_diff>
--- a/invoice_extractor/templates/material_requisition_template.xlsx
+++ b/invoice_extractor/templates/material_requisition_template.xlsx
@@ -438,7 +438,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="128">
+  <cellXfs count="129">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -755,6 +755,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1563,7 +1566,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" s="102">
       <c r="B19" s="73" t="n"/>
-      <c r="C19" s="89" t="n"/>
+      <c r="C19" s="62" t="n"/>
       <c r="H19" s="78" t="n"/>
       <c r="K19" s="73" t="n"/>
       <c r="L19" s="68" t="n"/>
@@ -1571,7 +1574,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" s="102">
       <c r="B20" s="20" t="n"/>
-      <c r="C20" s="81" t="n"/>
+      <c r="C20" s="64" t="n"/>
       <c r="G20" s="114" t="n"/>
       <c r="H20" s="115" t="n"/>
       <c r="J20" s="114" t="n"/>
@@ -1582,7 +1585,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" s="102">
       <c r="B21" s="20" t="n"/>
-      <c r="C21" s="81" t="n"/>
+      <c r="C21" s="64" t="n"/>
       <c r="G21" s="114" t="n"/>
       <c r="H21" s="115" t="n"/>
       <c r="J21" s="114" t="n"/>
@@ -1777,7 +1780,7 @@
     </row>
     <row r="40" ht="19.5" customHeight="1" s="102" thickBot="1">
       <c r="B40" s="27" t="n"/>
-      <c r="C40" s="121" t="n"/>
+      <c r="C40" s="128" t="n"/>
       <c r="D40" s="122" t="n"/>
       <c r="E40" s="122" t="n"/>
       <c r="F40" s="122" t="n"/>

</xml_diff>

<commit_message>
Embed Mohd Lukman signature into Material Requisition template
</commit_message>
<xml_diff>
--- a/invoice_extractor/templates/material_requisition_template.xlsx
+++ b/invoice_extractor/templates/material_requisition_template.xlsx
@@ -1014,6 +1014,31 @@
     </pic>
     <clientData/>
   </twoCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1333500" cy="809625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 

</xml_diff>

<commit_message>
Embed exact Mohd Lukman signature from reference MR template
</commit_message>
<xml_diff>
--- a/invoice_extractor/templates/material_requisition_template.xlsx
+++ b/invoice_extractor/templates/material_requisition_template.xlsx
@@ -438,7 +438,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -755,9 +755,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1018,10 +1015,10 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>47</row>
+      <row>45</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1333500" cy="809625"/>
+    <ext cx="1428750" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -1591,7 +1588,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" s="102">
       <c r="B19" s="73" t="n"/>
-      <c r="C19" s="62" t="n"/>
+      <c r="C19" s="89" t="n"/>
       <c r="H19" s="78" t="n"/>
       <c r="K19" s="73" t="n"/>
       <c r="L19" s="68" t="n"/>
@@ -1599,7 +1596,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" s="102">
       <c r="B20" s="20" t="n"/>
-      <c r="C20" s="64" t="n"/>
+      <c r="C20" s="81" t="n"/>
       <c r="G20" s="114" t="n"/>
       <c r="H20" s="115" t="n"/>
       <c r="J20" s="114" t="n"/>
@@ -1610,7 +1607,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" s="102">
       <c r="B21" s="20" t="n"/>
-      <c r="C21" s="64" t="n"/>
+      <c r="C21" s="81" t="n"/>
       <c r="G21" s="114" t="n"/>
       <c r="H21" s="115" t="n"/>
       <c r="J21" s="114" t="n"/>
@@ -1805,7 +1802,7 @@
     </row>
     <row r="40" ht="19.5" customHeight="1" s="102" thickBot="1">
       <c r="B40" s="27" t="n"/>
-      <c r="C40" s="128" t="n"/>
+      <c r="C40" s="121" t="n"/>
       <c r="D40" s="122" t="n"/>
       <c r="E40" s="122" t="n"/>
       <c r="F40" s="122" t="n"/>

</xml_diff>